<commit_message>
estamos, quedo todo listo
</commit_message>
<xml_diff>
--- a/live_report_SMC_HYPEUSDT.xlsx
+++ b/live_report_SMC_HYPEUSDT.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -886,6 +886,68 @@
       </c>
       <c r="P7" t="n">
         <v>51.12748134289693</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-11-13</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>21:30:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-11-15</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>14:08:53</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>38.294</v>
+      </c>
+      <c r="G8" t="n">
+        <v>38.5442625</v>
+      </c>
+      <c r="H8" t="n">
+        <v>38.5442625</v>
+      </c>
+      <c r="I8" t="n">
+        <v>37.33665</v>
+      </c>
+      <c r="J8" t="n">
+        <v>40.71928666666666</v>
+      </c>
+      <c r="K8" t="n">
+        <v>12.4267366365042</v>
+      </c>
+      <c r="L8" t="n">
+        <v>475.8694527582916</v>
+      </c>
+      <c r="M8" t="n">
+        <v>31.72463018388611</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>-3.109946177493195</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>SMC Stop Loss</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>59.08897737237071</v>
       </c>
     </row>
   </sheetData>

</xml_diff>